<commit_message>
update requirements.txt, compute area in mm^2
</commit_message>
<xml_diff>
--- a/local/P1466_P1365_Contraction_videos_legend.xlsx
+++ b/local/P1466_P1365_Contraction_videos_legend.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donatella.cea/Documents/Contraction analysis of neuromuscular organoids/NMOs-Contraction/local/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDE97495-23E9-D045-877D-05F4399A0DA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7617B080-8ADA-7A41-B97A-E7CF3C09A3F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35160" yWindow="-720" windowWidth="28800" windowHeight="16520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33140" yWindow="-860" windowWidth="28800" windowHeight="16520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="171">
   <si>
     <t>Video name</t>
   </si>
@@ -512,6 +512,27 @@
   </si>
   <si>
     <t>P1365_SMA_BRAN_d58_O4_c_3</t>
+  </si>
+  <si>
+    <t>Energy</t>
+  </si>
+  <si>
+    <t>Mean</t>
+  </si>
+  <si>
+    <t>%_of_count_above_threshold</t>
+  </si>
+  <si>
+    <t>%_of_absolute_sum_of_changes</t>
+  </si>
+  <si>
+    <t>Quantile_75</t>
+  </si>
+  <si>
+    <t>Standard_deviation</t>
+  </si>
+  <si>
+    <t>%_of_count_above_mean</t>
   </si>
 </sst>
 </file>
@@ -875,10 +896,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R133"/>
+  <dimension ref="A1:Y133"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="26.5" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -933,8 +957,29 @@
       <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S1" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -974,11 +1019,14 @@
       <c r="P2">
         <v>1</v>
       </c>
+      <c r="Q2">
+        <v>56</v>
+      </c>
       <c r="R2">
         <v>0.54</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -1018,11 +1066,14 @@
       <c r="P3">
         <v>1</v>
       </c>
+      <c r="Q3">
+        <v>55</v>
+      </c>
       <c r="R3">
         <v>0.64</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -1062,11 +1113,14 @@
       <c r="P4">
         <v>1</v>
       </c>
+      <c r="Q4">
+        <v>40</v>
+      </c>
       <c r="R4">
         <v>0.64</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -1106,11 +1160,14 @@
       <c r="P5">
         <v>1</v>
       </c>
+      <c r="Q5">
+        <v>60</v>
+      </c>
       <c r="R5">
         <v>0.64</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -1150,11 +1207,14 @@
       <c r="P6">
         <v>1</v>
       </c>
+      <c r="Q6">
+        <v>70</v>
+      </c>
       <c r="R6">
         <v>0.64</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -1194,11 +1254,14 @@
       <c r="P7">
         <v>1</v>
       </c>
+      <c r="Q7">
+        <v>50</v>
+      </c>
       <c r="R7">
         <v>0.63</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -1238,11 +1301,14 @@
       <c r="P8">
         <v>1</v>
       </c>
+      <c r="Q8">
+        <v>55</v>
+      </c>
       <c r="R8">
         <v>0.63</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -1282,11 +1348,14 @@
       <c r="P9">
         <v>1</v>
       </c>
+      <c r="Q9">
+        <v>55</v>
+      </c>
       <c r="R9">
         <v>0.61</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -1326,11 +1395,14 @@
       <c r="P10">
         <v>1</v>
       </c>
+      <c r="Q10">
+        <v>55</v>
+      </c>
       <c r="R10">
         <v>0.7</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>34</v>
       </c>
@@ -1370,11 +1442,14 @@
       <c r="P11">
         <v>1</v>
       </c>
+      <c r="Q11">
+        <v>55</v>
+      </c>
       <c r="R11">
         <v>0.72</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>35</v>
       </c>
@@ -1414,11 +1489,14 @@
       <c r="P12">
         <v>1</v>
       </c>
+      <c r="Q12">
+        <v>55</v>
+      </c>
       <c r="R12">
         <v>0.65</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>36</v>
       </c>
@@ -1458,11 +1536,14 @@
       <c r="P13">
         <v>1</v>
       </c>
+      <c r="Q13">
+        <v>55</v>
+      </c>
       <c r="R13">
         <v>0.66</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -1502,11 +1583,14 @@
       <c r="P14">
         <v>1</v>
       </c>
+      <c r="Q14">
+        <v>55</v>
+      </c>
       <c r="R14">
         <v>0.66</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>39</v>
       </c>
@@ -1546,11 +1630,14 @@
       <c r="P15">
         <v>1</v>
       </c>
+      <c r="Q15">
+        <v>55</v>
+      </c>
       <c r="R15">
         <v>0.67</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>40</v>
       </c>
@@ -1589,6 +1676,9 @@
       </c>
       <c r="P16">
         <v>1</v>
+      </c>
+      <c r="Q16">
+        <v>55</v>
       </c>
       <c r="R16">
         <v>0.65</v>
@@ -1634,6 +1724,9 @@
       <c r="P17">
         <v>1</v>
       </c>
+      <c r="Q17">
+        <v>55</v>
+      </c>
       <c r="R17">
         <v>0.72</v>
       </c>
@@ -1678,6 +1771,9 @@
       <c r="P18">
         <v>1</v>
       </c>
+      <c r="Q18">
+        <v>60</v>
+      </c>
       <c r="R18">
         <v>0.67</v>
       </c>
@@ -1722,6 +1818,9 @@
       <c r="P19">
         <v>1</v>
       </c>
+      <c r="Q19">
+        <v>60</v>
+      </c>
       <c r="R19">
         <v>0.63</v>
       </c>
@@ -1766,6 +1865,9 @@
       <c r="P20">
         <v>1</v>
       </c>
+      <c r="Q20">
+        <v>60</v>
+      </c>
       <c r="R20">
         <v>0.59</v>
       </c>
@@ -1810,6 +1912,9 @@
       <c r="P21">
         <v>1</v>
       </c>
+      <c r="Q21">
+        <v>60</v>
+      </c>
       <c r="R21">
         <v>0.64</v>
       </c>
@@ -1854,6 +1959,9 @@
       <c r="P22">
         <v>1</v>
       </c>
+      <c r="Q22">
+        <v>60</v>
+      </c>
       <c r="R22">
         <v>0.65</v>
       </c>
@@ -1898,6 +2006,9 @@
       <c r="P23">
         <v>1</v>
       </c>
+      <c r="Q23">
+        <v>60</v>
+      </c>
       <c r="R23">
         <v>0.66</v>
       </c>
@@ -1942,6 +2053,9 @@
       <c r="P24">
         <v>1</v>
       </c>
+      <c r="Q24">
+        <v>60</v>
+      </c>
       <c r="R24">
         <v>0.65</v>
       </c>
@@ -1986,6 +2100,9 @@
       <c r="P25">
         <v>1</v>
       </c>
+      <c r="Q25">
+        <v>60</v>
+      </c>
       <c r="R25">
         <v>0.65</v>
       </c>
@@ -2030,6 +2147,9 @@
       <c r="P26">
         <v>1</v>
       </c>
+      <c r="Q26">
+        <v>60</v>
+      </c>
       <c r="R26">
         <v>0.63</v>
       </c>
@@ -2074,6 +2194,9 @@
       <c r="P27">
         <v>1</v>
       </c>
+      <c r="Q27">
+        <v>60</v>
+      </c>
       <c r="R27">
         <v>0.61</v>
       </c>
@@ -4836,5 +4959,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>